<commit_message>
update real constants excel
</commit_message>
<xml_diff>
--- a/tests/3D_loop_cond_base/input_template.xlsx
+++ b/tests/3D_loop_cond_base/input_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PlasmaArc\simulations\3D_loop_cond_base\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PlasmaArc\tests\3D_loop_cond_base\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE2681C8-2D9E-4CFC-9760-9D7841987FFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C2FDACA-EF59-4F38-850B-1686826996AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1275" yWindow="1275" windowWidth="18000" windowHeight="9360" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="element_types" sheetId="1" r:id="rId1"/>
@@ -1278,7 +1278,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:W1"/>
+  <dimension ref="A1:W2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.140625" bestFit="1" customWidth="1"/>
@@ -1355,6 +1355,77 @@
       </c>
       <c r="W1" t="s">
         <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
+      <c r="Q2">
+        <v>0</v>
+      </c>
+      <c r="R2">
+        <v>0</v>
+      </c>
+      <c r="S2">
+        <v>0</v>
+      </c>
+      <c r="T2">
+        <v>0</v>
+      </c>
+      <c r="U2">
+        <v>0</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>